<commit_message>
@ v52/v53: 15/09 - TAKAMTSING 51282 retiree de §14 (repasse non planifiee), remplacee par BOUKAR ISAIE SO2604-52017 (3 100, BELGO-BERI Littoral minime, Payee). Plan v53 : 60 100/57 500 (11/09 107%, 15/09 103% +1 150, 8 forcees).
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prog poussin/Popo/output/Plan_Livraisons_BELGO_Ponte.xlsx
+++ b/Prog poussin/Popo/output/Plan_Livraisons_BELGO_Ponte.xlsx
@@ -936,7 +936,7 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Mar 15/09/2026 — Production: 37,500 | Region: Centre | Place libre: 0</t>
+          <t>Mar 15/09/2026 — Production: 37,500 | Region: Centre + Littoral | Place libre: 0 [Littoral minime: 3,100 (ÉCHUE: 3,100)]</t>
         </is>
       </c>
       <c r="C12" s="4" t="n"/>
@@ -1426,12 +1426,12 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>TAKAMTSING PROSPER</t>
+          <t>BOUKAR ISAIE</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>SO2604-51282</t>
+          <t>SO2604-52017</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1440,34 +1440,34 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>5800</v>
+        <v>3100</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>5800</v>
+        <v>3100</v>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>BELGO-NKOABANG</t>
+          <t>BELGO-BERI</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>165 j</t>
+          <t>158 j</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>12/09/2026</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
@@ -1491,7 +1491,7 @@
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="6" t="n">
-        <v>41350</v>
+        <v>38650</v>
       </c>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n"/>
@@ -1512,7 +1512,7 @@
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="8" t="n">
-        <v>62800</v>
+        <v>60100</v>
       </c>
       <c r="G23" s="9" t="n"/>
       <c r="H23" s="9" t="n"/>
@@ -2154,7 +2154,7 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Mar 15/09/2026 — Production: 35,650 | Region: Centre | Place libre: 0</t>
+          <t>Mar 15/09/2026 — Production: 35,650 | Region: Centre + Littoral | Place libre: 0 [Littoral minime: 3,100 (ÉCHUE: 3,100)]</t>
         </is>
       </c>
       <c r="C12" s="4" t="n"/>
@@ -2644,12 +2644,12 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>TAKAMTSING PROSPER</t>
+          <t>BOUKAR ISAIE</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>SO2604-51282</t>
+          <t>SO2604-52017</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -2658,34 +2658,34 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>5800</v>
+        <v>3100</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>5800</v>
+        <v>3100</v>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>BELGO-NKOABANG</t>
+          <t>BELGO-BERI</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>165 j</t>
+          <t>158 j</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>12/09/2026</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
@@ -2709,7 +2709,7 @@
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="6" t="n">
-        <v>41350</v>
+        <v>38650</v>
       </c>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n"/>
@@ -2730,7 +2730,7 @@
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="8" t="n">
-        <v>62800</v>
+        <v>60100</v>
       </c>
       <c r="G23" s="9" t="n"/>
       <c r="H23" s="9" t="n"/>
@@ -4019,19 +4019,19 @@
     <row r="31">
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>SANDJONG ELIE</t>
+          <t>TAKAMTSING PROSPER</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>SO2604-51281</t>
+          <t>SO2604-51282</t>
         </is>
       </c>
       <c r="D31" s="15" t="n">
-        <v>2200</v>
+        <v>5800</v>
       </c>
       <c r="E31" s="15" t="n">
-        <v>2200</v>
+        <v>5800</v>
       </c>
       <c r="F31" s="15" t="inlineStr">
         <is>
@@ -4057,28 +4057,28 @@
     <row r="32">
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>PANEBENG VICTOR DG</t>
+          <t>SANDJONG ELIE</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67892</t>
+          <t>SO2604-51281</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>30000</v>
+        <v>2200</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>30000</v>
+        <v>2200</v>
       </c>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G32" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-NKOABANG</t>
         </is>
       </c>
       <c r="H32" s="15" t="inlineStr">
@@ -4088,35 +4088,35 @@
       </c>
       <c r="I32" s="15" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>KENNE TCHUENTE JILDAS ANICET</t>
+          <t>PANEBENG VICTOR DG</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>SO2604-51270</t>
+          <t>SO2608-67892</t>
         </is>
       </c>
       <c r="D33" s="15" t="n">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="E33" s="15" t="n">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H33" s="15" t="inlineStr">
@@ -4133,28 +4133,28 @@
     <row r="34">
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>Tezingang Fomo Gabriel</t>
+          <t>KENNE TCHUENTE JILDAS ANICET</t>
         </is>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67697</t>
+          <t>SO2604-51270</t>
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>25000</v>
+        <v>3000</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>25000</v>
+        <v>3000</v>
       </c>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G34" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H34" s="15" t="inlineStr">
@@ -4164,19 +4164,19 @@
       </c>
       <c r="I34" s="15" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>26/08/2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>PANEBENG VICTOR DG</t>
+          <t>Tezingang Fomo Gabriel</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67890</t>
+          <t>SO2608-67697</t>
         </is>
       </c>
       <c r="D35" s="15" t="n">
@@ -4209,19 +4209,19 @@
     <row r="36">
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>NOUBO KENFACK EVELINE</t>
+          <t>PANEBENG VICTOR DG</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66752</t>
+          <t>SO2608-67890</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>6000</v>
+        <v>25000</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>6000</v>
+        <v>25000</v>
       </c>
       <c r="F36" s="15" t="inlineStr">
         <is>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G36" s="15" t="inlineStr">
         <is>
-          <t>BELGO MBOUDA</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H36" s="15" t="inlineStr">
@@ -4247,19 +4247,19 @@
     <row r="37">
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>TCHINDA KAAWE SOL PLEISIS</t>
+          <t>NOUBO KENFACK EVELINE</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66806</t>
+          <t>SO2608-66752</t>
         </is>
       </c>
       <c r="D37" s="15" t="n">
-        <v>2400</v>
+        <v>6000</v>
       </c>
       <c r="E37" s="15" t="n">
-        <v>2400</v>
+        <v>6000</v>
       </c>
       <c r="F37" s="15" t="inlineStr">
         <is>
@@ -4268,7 +4268,7 @@
       </c>
       <c r="G37" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO MBOUDA</t>
         </is>
       </c>
       <c r="H37" s="15" t="inlineStr">
@@ -4285,19 +4285,19 @@
     <row r="38">
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>SAGUEN DEFFO CHANCELIER RICHARD</t>
+          <t>TCHINDA KAAWE SOL PLEISIS</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68306</t>
+          <t>SO2608-66806</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>30000</v>
+        <v>2400</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>30000</v>
+        <v>2400</v>
       </c>
       <c r="F38" s="15" t="inlineStr">
         <is>
@@ -4316,26 +4316,26 @@
       </c>
       <c r="I38" s="15" t="inlineStr">
         <is>
-          <t>29/08/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>PANEBENG VICTOR DG</t>
+          <t>SAGUEN DEFFO CHANCELIER RICHARD</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67889</t>
+          <t>SO2608-68306</t>
         </is>
       </c>
       <c r="D39" s="15" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="E39" s="15" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="F39" s="15" t="inlineStr">
         <is>
@@ -4361,19 +4361,19 @@
     <row r="40">
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>TCHINDA KAAWE SOL PLEISIS</t>
+          <t>PANEBENG VICTOR DG</t>
         </is>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66802</t>
+          <t>SO2608-67889</t>
         </is>
       </c>
       <c r="D40" s="15" t="n">
-        <v>9000</v>
+        <v>25000</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>9000</v>
+        <v>25000</v>
       </c>
       <c r="F40" s="15" t="inlineStr">
         <is>
@@ -4399,19 +4399,19 @@
     <row r="41">
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>OUMAROU BOBBO ISSA</t>
+          <t>TCHINDA KAAWE SOL PLEISIS</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66755</t>
+          <t>SO2608-66802</t>
         </is>
       </c>
       <c r="D41" s="15" t="n">
-        <v>4000</v>
+        <v>9000</v>
       </c>
       <c r="E41" s="15" t="n">
-        <v>4000</v>
+        <v>9000</v>
       </c>
       <c r="F41" s="15" t="inlineStr">
         <is>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="G41" s="15" t="inlineStr">
         <is>
-          <t>BELGO MBOUDA</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H41" s="15" t="inlineStr">
@@ -4437,19 +4437,19 @@
     <row r="42">
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>LEMNYUY BETILLA</t>
+          <t>OUMAROU BOBBO ISSA</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66754</t>
+          <t>SO2608-66755</t>
         </is>
       </c>
       <c r="D42" s="15" t="n">
-        <v>3400</v>
+        <v>4000</v>
       </c>
       <c r="E42" s="15" t="n">
-        <v>3400</v>
+        <v>4000</v>
       </c>
       <c r="F42" s="15" t="inlineStr">
         <is>
@@ -4475,19 +4475,19 @@
     <row r="43">
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>Biepip Ngoufo Dolf Brice</t>
+          <t>LEMNYUY BETILLA</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60194</t>
+          <t>SO2608-66754</t>
         </is>
       </c>
       <c r="D43" s="15" t="n">
-        <v>7800</v>
+        <v>3400</v>
       </c>
       <c r="E43" s="15" t="n">
-        <v>7800</v>
+        <v>3400</v>
       </c>
       <c r="F43" s="15" t="inlineStr">
         <is>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="G43" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDJELENG</t>
+          <t>BELGO MBOUDA</t>
         </is>
       </c>
       <c r="H43" s="15" t="inlineStr">
@@ -4513,19 +4513,19 @@
     <row r="44">
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>FOTSO LEODOR</t>
+          <t>Biepip Ngoufo Dolf Brice</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60971</t>
+          <t>SO2606-60194</t>
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>4400</v>
+        <v>7800</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>4400</v>
+        <v>7800</v>
       </c>
       <c r="F44" s="15" t="inlineStr">
         <is>
@@ -4551,28 +4551,28 @@
     <row r="45">
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>PIEBJOU MICHEL</t>
+          <t>FOTSO LEODOR</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>SO2604-51756</t>
+          <t>SO2606-60971</t>
         </is>
       </c>
       <c r="D45" s="15" t="n">
-        <v>2100</v>
+        <v>4400</v>
       </c>
       <c r="E45" s="15" t="n">
-        <v>2100</v>
+        <v>4400</v>
       </c>
       <c r="F45" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G45" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NKOABANG</t>
+          <t>BELGO-NDJELENG</t>
         </is>
       </c>
       <c r="H45" s="15" t="inlineStr">
@@ -4589,28 +4589,28 @@
     <row r="46">
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>Wokam Kunatse Raymond</t>
+          <t>PIEBJOU MICHEL</t>
         </is>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68148</t>
+          <t>SO2604-51756</t>
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>11000</v>
+        <v>2100</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>11000</v>
+        <v>2100</v>
       </c>
       <c r="F46" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G46" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-NKOABANG</t>
         </is>
       </c>
       <c r="H46" s="15" t="inlineStr">
@@ -4620,26 +4620,26 @@
       </c>
       <c r="I46" s="15" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>29/08/2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>First Agriculture &amp; Elevage Sarl (F.a.e Sarl)</t>
+          <t>Wokam Kunatse Raymond</t>
         </is>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68068</t>
+          <t>SO2608-68148</t>
         </is>
       </c>
       <c r="D47" s="15" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="E47" s="15" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="F47" s="15" t="inlineStr">
         <is>
@@ -4665,19 +4665,19 @@
     <row r="48">
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>GIC CHRETIENS</t>
+          <t>First Agriculture &amp; Elevage Sarl (F.a.e Sarl)</t>
         </is>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68271</t>
+          <t>SO2608-68068</t>
         </is>
       </c>
       <c r="D48" s="15" t="n">
-        <v>6000</v>
+        <v>10000</v>
       </c>
       <c r="E48" s="15" t="n">
-        <v>6000</v>
+        <v>10000</v>
       </c>
       <c r="F48" s="15" t="inlineStr">
         <is>
@@ -4696,35 +4696,35 @@
       </c>
       <c r="I48" s="15" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>Ngouadjeu Paul</t>
+          <t>GIC CHRETIENS</t>
         </is>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>SO2605-56216</t>
+          <t>SO2608-68271</t>
         </is>
       </c>
       <c r="D49" s="15" t="n">
-        <v>3300</v>
+        <v>6000</v>
       </c>
       <c r="E49" s="15" t="n">
-        <v>3300</v>
+        <v>6000</v>
       </c>
       <c r="F49" s="15" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G49" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NKONGSAMBA</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H49" s="15" t="inlineStr">
@@ -4741,28 +4741,28 @@
     <row r="50">
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>TUMENTA  GRACE</t>
+          <t>Ngouadjeu Paul</t>
         </is>
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>SO2604-53701</t>
+          <t>SO2605-56216</t>
         </is>
       </c>
       <c r="D50" s="15" t="n">
-        <v>2000</v>
+        <v>3300</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>2000</v>
+        <v>3300</v>
       </c>
       <c r="F50" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="G50" s="15" t="inlineStr">
         <is>
-          <t>BELGO MBOUDA</t>
+          <t>BELGO-NKONGSAMBA</t>
         </is>
       </c>
       <c r="H50" s="15" t="inlineStr">
@@ -4779,19 +4779,19 @@
     <row r="51">
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>Tengemne Gniteyo Steve</t>
+          <t>TUMENTA  GRACE</t>
         </is>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68577</t>
+          <t>SO2604-53701</t>
         </is>
       </c>
       <c r="D51" s="15" t="n">
-        <v>25000</v>
+        <v>2000</v>
       </c>
       <c r="E51" s="15" t="n">
-        <v>25000</v>
+        <v>2000</v>
       </c>
       <c r="F51" s="15" t="inlineStr">
         <is>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="G51" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO MBOUDA</t>
         </is>
       </c>
       <c r="H51" s="15" t="inlineStr">
@@ -4810,26 +4810,26 @@
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>04/09/2026</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="15" t="inlineStr">
         <is>
-          <t>Fotie Tagoumtse Constantin Legrand</t>
+          <t>Tengemne Gniteyo Steve</t>
         </is>
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68336</t>
+          <t>SO2609-68577</t>
         </is>
       </c>
       <c r="D52" s="15" t="n">
-        <v>10500</v>
+        <v>25000</v>
       </c>
       <c r="E52" s="15" t="n">
-        <v>10500</v>
+        <v>25000</v>
       </c>
       <c r="F52" s="15" t="inlineStr">
         <is>
@@ -4855,19 +4855,19 @@
     <row r="53">
       <c r="B53" s="15" t="inlineStr">
         <is>
-          <t>FOTSO KAMGA</t>
+          <t>Fotie Tagoumtse Constantin Legrand</t>
         </is>
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68683</t>
+          <t>SO2608-68336</t>
         </is>
       </c>
       <c r="D53" s="15" t="n">
-        <v>5000</v>
+        <v>10500</v>
       </c>
       <c r="E53" s="15" t="n">
-        <v>5000</v>
+        <v>10500</v>
       </c>
       <c r="F53" s="15" t="inlineStr">
         <is>
@@ -4893,12 +4893,12 @@
     <row r="54">
       <c r="B54" s="15" t="inlineStr">
         <is>
-          <t>TAMDJOZAM TALLAH PHRIXOS STALINE</t>
+          <t>FOTSO KAMGA</t>
         </is>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68474</t>
+          <t>SO2609-68683</t>
         </is>
       </c>
       <c r="D54" s="15" t="n">
@@ -4931,19 +4931,19 @@
     <row r="55">
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>Tengemne Gniteyo Steve</t>
+          <t>TAMDJOZAM TALLAH PHRIXOS STALINE</t>
         </is>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68586</t>
+          <t>SO2608-68474</t>
         </is>
       </c>
       <c r="D55" s="15" t="n">
-        <v>12000</v>
+        <v>5000</v>
       </c>
       <c r="E55" s="15" t="n">
-        <v>12000</v>
+        <v>5000</v>
       </c>
       <c r="F55" s="15" t="inlineStr">
         <is>
@@ -4962,26 +4962,26 @@
       </c>
       <c r="I55" s="15" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>FIRST AGRICULTURE ET ELEVAGE SARL</t>
+          <t>Tengemne Gniteyo Steve</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68680</t>
+          <t>SO2609-68586</t>
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="F56" s="15" t="inlineStr">
         <is>
@@ -5007,19 +5007,19 @@
     <row r="57">
       <c r="B57" s="15" t="inlineStr">
         <is>
-          <t>MERAUDE BILOA MISSE MARCELINE FELICITE</t>
+          <t>FIRST AGRICULTURE ET ELEVAGE SARL</t>
         </is>
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68086</t>
+          <t>SO2609-68680</t>
         </is>
       </c>
       <c r="D57" s="15" t="n">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="E57" s="15" t="n">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="F57" s="15" t="inlineStr">
         <is>
@@ -5045,19 +5045,19 @@
     <row r="58">
       <c r="B58" s="15" t="inlineStr">
         <is>
-          <t>SONWA RONICE BERTHOL</t>
+          <t>MERAUDE BILOA MISSE MARCELINE FELICITE</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68067</t>
+          <t>SO2608-68086</t>
         </is>
       </c>
       <c r="D58" s="15" t="n">
-        <v>1100</v>
+        <v>4000</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>1100</v>
+        <v>4000</v>
       </c>
       <c r="F58" s="15" t="inlineStr">
         <is>
@@ -5083,19 +5083,19 @@
     <row r="59">
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>Tengemne Gniteyo Steve</t>
+          <t>SONWA RONICE BERTHOL</t>
         </is>
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68585</t>
+          <t>SO2608-68067</t>
         </is>
       </c>
       <c r="D59" s="15" t="n">
-        <v>13000</v>
+        <v>1100</v>
       </c>
       <c r="E59" s="15" t="n">
-        <v>13000</v>
+        <v>1100</v>
       </c>
       <c r="F59" s="15" t="inlineStr">
         <is>
@@ -5114,26 +5114,26 @@
       </c>
       <c r="I59" s="15" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="15" t="inlineStr">
         <is>
-          <t>DJUISSI FOKO CARMEN  (DJUISSI FOKO CARMEN )</t>
+          <t>Tengemne Gniteyo Steve</t>
         </is>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68591</t>
+          <t>SO2609-68585</t>
         </is>
       </c>
       <c r="D60" s="15" t="n">
-        <v>1000</v>
+        <v>13000</v>
       </c>
       <c r="E60" s="15" t="n">
-        <v>1000</v>
+        <v>13000</v>
       </c>
       <c r="F60" s="15" t="inlineStr">
         <is>
@@ -5152,26 +5152,26 @@
       </c>
       <c r="I60" s="15" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="15" t="inlineStr">
         <is>
-          <t>SECRET DE L'ELEVEUR</t>
+          <t>DJUISSI FOKO CARMEN  (DJUISSI FOKO CARMEN )</t>
         </is>
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68713</t>
+          <t>SO2609-68591</t>
         </is>
       </c>
       <c r="D61" s="15" t="n">
-        <v>5200</v>
+        <v>1000</v>
       </c>
       <c r="E61" s="15" t="n">
-        <v>5200</v>
+        <v>1000</v>
       </c>
       <c r="F61" s="15" t="inlineStr">
         <is>
@@ -5197,19 +5197,19 @@
     <row r="62">
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>TESEHKOUE CHARLES</t>
+          <t>SECRET DE L'ELEVEUR</t>
         </is>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>SO2606-61310</t>
+          <t>SO2609-68713</t>
         </is>
       </c>
       <c r="D62" s="15" t="n">
-        <v>10150</v>
+        <v>5200</v>
       </c>
       <c r="E62" s="15" t="n">
-        <v>10150</v>
+        <v>5200</v>
       </c>
       <c r="F62" s="15" t="inlineStr">
         <is>
@@ -5223,40 +5223,40 @@
       </c>
       <c r="H62" s="15" t="inlineStr">
         <is>
-          <t>ÉCHUE RECLASSÉE</t>
+          <t>ÉCHUE</t>
         </is>
       </c>
       <c r="I62" s="15" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" s="15" t="inlineStr">
         <is>
-          <t>Groupe D'initiative Commune Des Jeunes Producteurs Agropastoraux De L'est (Gic/Jepro-Agro)</t>
+          <t>TESEHKOUE CHARLES</t>
         </is>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>SO2605-55433</t>
+          <t>SO2606-61310</t>
         </is>
       </c>
       <c r="D63" s="15" t="n">
-        <v>6500</v>
+        <v>10150</v>
       </c>
       <c r="E63" s="15" t="n">
-        <v>6500</v>
+        <v>10150</v>
       </c>
       <c r="F63" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G63" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H63" s="15" t="inlineStr">
@@ -5266,26 +5266,26 @@
       </c>
       <c r="I63" s="15" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>08/07/2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>MB Reference SARL (Moiffo Pascal Blaise)</t>
+          <t>Groupe D'initiative Commune Des Jeunes Producteurs Agropastoraux De L'est (Gic/Jepro-Agro)</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>SO2607-62336</t>
+          <t>SO2605-55433</t>
         </is>
       </c>
       <c r="D64" s="15" t="n">
-        <v>13100</v>
+        <v>6500</v>
       </c>
       <c r="E64" s="15" t="n">
-        <v>13100</v>
+        <v>6500</v>
       </c>
       <c r="F64" s="15" t="inlineStr">
         <is>
@@ -5304,35 +5304,35 @@
       </c>
       <c r="I64" s="15" t="inlineStr">
         <is>
-          <t>21/07/2026</t>
+          <t>15/07/2026</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>Kenne Manfouo Idrice</t>
+          <t>MB Reference SARL (Moiffo Pascal Blaise)</t>
         </is>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>SO2605-57744</t>
+          <t>SO2607-62336</t>
         </is>
       </c>
       <c r="D65" s="15" t="n">
-        <v>16000</v>
+        <v>13100</v>
       </c>
       <c r="E65" s="15" t="n">
-        <v>16000</v>
+        <v>13100</v>
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G65" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDJELENG</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H65" s="15" t="inlineStr">
@@ -5342,35 +5342,35 @@
       </c>
       <c r="I65" s="15" t="inlineStr">
         <is>
-          <t>25/07/2026</t>
+          <t>21/07/2026</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>KAMDEM MERLIN</t>
+          <t>Kenne Manfouo Idrice</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>SO2604-51411</t>
+          <t>SO2605-57744</t>
         </is>
       </c>
       <c r="D66" s="15" t="n">
-        <v>23000</v>
+        <v>16000</v>
       </c>
       <c r="E66" s="15" t="n">
-        <v>23000</v>
+        <v>16000</v>
       </c>
       <c r="F66" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G66" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-NDJELENG</t>
         </is>
       </c>
       <c r="H66" s="15" t="inlineStr">
@@ -5380,35 +5380,35 @@
       </c>
       <c r="I66" s="15" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>25/07/2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="15" t="inlineStr">
         <is>
-          <t>TCHEUMTCHOUA DANIEL</t>
+          <t>KAMDEM MERLIN</t>
         </is>
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68048</t>
+          <t>SO2604-51411</t>
         </is>
       </c>
       <c r="D67" s="15" t="n">
-        <v>11000</v>
+        <v>23000</v>
       </c>
       <c r="E67" s="15" t="n">
-        <v>11000</v>
+        <v>23000</v>
       </c>
       <c r="F67" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G67" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H67" s="15" t="inlineStr">
@@ -5418,26 +5418,26 @@
       </c>
       <c r="I67" s="15" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>04/09/2026</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="15" t="inlineStr">
         <is>
-          <t>PRODIPEL SARL</t>
+          <t>TCHEUMTCHOUA DANIEL</t>
         </is>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68037</t>
+          <t>SO2608-68048</t>
         </is>
       </c>
       <c r="D68" s="15" t="n">
-        <v>18000</v>
+        <v>11000</v>
       </c>
       <c r="E68" s="15" t="n">
-        <v>18000</v>
+        <v>11000</v>
       </c>
       <c r="F68" s="15" t="inlineStr">
         <is>
@@ -5456,73 +5456,73 @@
       </c>
       <c r="I68" s="15" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="15" t="inlineStr">
         <is>
-          <t>YFOU JASINO PEGUY</t>
+          <t>PRODIPEL SARL</t>
         </is>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>SO2604-51904</t>
+          <t>SO2608-68037</t>
         </is>
       </c>
       <c r="D69" s="15" t="n">
-        <v>23000</v>
+        <v>18000</v>
       </c>
       <c r="E69" s="15" t="n">
-        <v>23000</v>
+        <v>18000</v>
       </c>
       <c r="F69" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G69" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H69" s="15" t="inlineStr">
         <is>
-          <t>RECLASSÉE</t>
+          <t>ÉCHUE RECLASSÉE</t>
         </is>
       </c>
       <c r="I69" s="15" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="15" t="inlineStr">
         <is>
-          <t>MIAKAUG EPSE SODEA DIANE</t>
+          <t>YFOU JASINO PEGUY</t>
         </is>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66550</t>
+          <t>SO2604-51904</t>
         </is>
       </c>
       <c r="D70" s="15" t="n">
-        <v>1000</v>
+        <v>23000</v>
       </c>
       <c r="E70" s="15" t="n">
-        <v>1000</v>
+        <v>23000</v>
       </c>
       <c r="F70" s="15" t="inlineStr">
         <is>
-          <t>Nord</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G70" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDERE</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H70" s="15" t="inlineStr">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="I70" s="15" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
@@ -5544,14 +5544,14 @@
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66553</t>
+          <t>SO2608-66550</t>
         </is>
       </c>
       <c r="D71" s="15" t="n">
-        <v>1800</v>
+        <v>1000</v>
       </c>
       <c r="E71" s="15" t="n">
-        <v>1800</v>
+        <v>1000</v>
       </c>
       <c r="F71" s="15" t="inlineStr">
         <is>
@@ -5582,14 +5582,14 @@
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66552</t>
+          <t>SO2608-66553</t>
         </is>
       </c>
       <c r="D72" s="15" t="n">
-        <v>1400</v>
+        <v>1800</v>
       </c>
       <c r="E72" s="15" t="n">
-        <v>1400</v>
+        <v>1800</v>
       </c>
       <c r="F72" s="15" t="inlineStr">
         <is>
@@ -5620,14 +5620,14 @@
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66549</t>
+          <t>SO2608-66552</t>
         </is>
       </c>
       <c r="D73" s="15" t="n">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="E73" s="15" t="n">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="F73" s="15" t="inlineStr">
         <is>
@@ -5653,28 +5653,28 @@
     <row r="74">
       <c r="B74" s="15" t="inlineStr">
         <is>
-          <t>TEDONGMO ZOYIM AGOSTINI</t>
+          <t>MIAKAUG EPSE SODEA DIANE</t>
         </is>
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>SO2606-59043</t>
+          <t>SO2608-66549</t>
         </is>
       </c>
       <c r="D74" s="15" t="n">
-        <v>3200</v>
+        <v>1200</v>
       </c>
       <c r="E74" s="15" t="n">
-        <v>3200</v>
+        <v>1200</v>
       </c>
       <c r="F74" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Nord</t>
         </is>
       </c>
       <c r="G74" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-NDERE</t>
         </is>
       </c>
       <c r="H74" s="15" t="inlineStr">
@@ -5691,28 +5691,28 @@
     <row r="75">
       <c r="B75" s="15" t="inlineStr">
         <is>
-          <t>MOFFO FOBOU MERLIN (MOFFO FOBOU MERLIN)</t>
+          <t>TEDONGMO ZOYIM AGOSTINI</t>
         </is>
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>SO2606-59829</t>
+          <t>SO2606-59043</t>
         </is>
       </c>
       <c r="D75" s="15" t="n">
-        <v>5600</v>
+        <v>3200</v>
       </c>
       <c r="E75" s="15" t="n">
-        <v>5600</v>
+        <v>3200</v>
       </c>
       <c r="F75" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G75" s="15" t="inlineStr">
         <is>
-          <t>BELGO AHALA</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H75" s="15" t="inlineStr">
@@ -5722,35 +5722,35 @@
       </c>
       <c r="I75" s="15" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="15" t="inlineStr">
         <is>
-          <t>KENNY PATRICK</t>
+          <t>MOFFO FOBOU MERLIN (MOFFO FOBOU MERLIN)</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>SO2603-50649</t>
+          <t>SO2606-59829</t>
         </is>
       </c>
       <c r="D76" s="15" t="n">
-        <v>3500</v>
+        <v>5600</v>
       </c>
       <c r="E76" s="15" t="n">
-        <v>3500</v>
+        <v>5600</v>
       </c>
       <c r="F76" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G76" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO AHALA</t>
         </is>
       </c>
       <c r="H76" s="15" t="inlineStr">
@@ -5760,35 +5760,35 @@
       </c>
       <c r="I76" s="15" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="15" t="inlineStr">
         <is>
-          <t>PROVENDERIE L' ASSURANCE</t>
+          <t>KENNY PATRICK</t>
         </is>
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>SO2607-64984</t>
+          <t>SO2603-50649</t>
         </is>
       </c>
       <c r="D77" s="15" t="n">
-        <v>9600</v>
+        <v>3500</v>
       </c>
       <c r="E77" s="15" t="n">
-        <v>9600</v>
+        <v>3500</v>
       </c>
       <c r="F77" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G77" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H77" s="15" t="inlineStr">
@@ -5798,26 +5798,26 @@
       </c>
       <c r="I77" s="15" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>TAMATIO</t>
+          <t>PROVENDERIE L' ASSURANCE</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68923</t>
+          <t>SO2607-64984</t>
         </is>
       </c>
       <c r="D78" s="15" t="n">
-        <v>27300</v>
+        <v>9600</v>
       </c>
       <c r="E78" s="15" t="n">
-        <v>27300</v>
+        <v>9600</v>
       </c>
       <c r="F78" s="15" t="inlineStr">
         <is>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="G78" s="15" t="inlineStr">
         <is>
-          <t>BELGO AHALA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H78" s="15" t="inlineStr">
@@ -5836,26 +5836,26 @@
       </c>
       <c r="I78" s="15" t="inlineStr">
         <is>
-          <t>06/01/2027</t>
+          <t>23/10/2026</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="15" t="inlineStr">
         <is>
-          <t>FOOD FOR ALL COMPLEXE SARL</t>
+          <t>TAMATIO</t>
         </is>
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69154</t>
+          <t>SO2608-68923</t>
         </is>
       </c>
       <c r="D79" s="15" t="n">
-        <v>5000</v>
+        <v>27300</v>
       </c>
       <c r="E79" s="15" t="n">
-        <v>5000</v>
+        <v>27300</v>
       </c>
       <c r="F79" s="15" t="inlineStr">
         <is>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="G79" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO AHALA</t>
         </is>
       </c>
       <c r="H79" s="15" t="inlineStr">
@@ -5874,26 +5874,26 @@
       </c>
       <c r="I79" s="15" t="inlineStr">
         <is>
-          <t>07/01/2027</t>
+          <t>06/01/2027</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="15" t="inlineStr">
         <is>
-          <t>Kemajou Dorette</t>
+          <t>FOOD FOR ALL COMPLEXE SARL</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60066</t>
+          <t>SO2609-69154</t>
         </is>
       </c>
       <c r="D80" s="15" t="n">
-        <v>1500</v>
+        <v>5000</v>
       </c>
       <c r="E80" s="15" t="n">
-        <v>1500</v>
+        <v>5000</v>
       </c>
       <c r="F80" s="15" t="inlineStr">
         <is>
@@ -5907,40 +5907,40 @@
       </c>
       <c r="H80" s="15" t="inlineStr">
         <is>
-          <t>IMMINENTE</t>
+          <t>RECLASSÉE</t>
         </is>
       </c>
       <c r="I80" s="15" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>07/01/2027</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" s="15" t="inlineStr">
         <is>
-          <t>TIADJOUE EMMANUEL</t>
+          <t>Kemajou Dorette</t>
         </is>
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>SO2607-63432</t>
+          <t>SO2606-60066</t>
         </is>
       </c>
       <c r="D81" s="15" t="n">
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="E81" s="15" t="n">
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="F81" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G81" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H81" s="15" t="inlineStr">
@@ -5950,26 +5950,26 @@
       </c>
       <c r="I81" s="15" t="inlineStr">
         <is>
-          <t>12/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>TEDOGMO ZOYIM AGOSTINI</t>
+          <t>TIADJOUE EMMANUEL</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69006</t>
+          <t>SO2607-63432</t>
         </is>
       </c>
       <c r="D82" s="15" t="n">
-        <v>6200</v>
+        <v>800</v>
       </c>
       <c r="E82" s="15" t="n">
-        <v>6200</v>
+        <v>800</v>
       </c>
       <c r="F82" s="15" t="inlineStr">
         <is>
@@ -5978,7 +5978,7 @@
       </c>
       <c r="G82" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDJELENG</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H82" s="15" t="inlineStr">
@@ -5995,19 +5995,19 @@
     <row r="83">
       <c r="B83" s="15" t="inlineStr">
         <is>
-          <t>KAMGANG EMMANUEL</t>
+          <t>TEDOGMO ZOYIM AGOSTINI</t>
         </is>
       </c>
       <c r="C83" s="15" t="inlineStr">
         <is>
-          <t>SO2606-58404</t>
+          <t>SO2609-69006</t>
         </is>
       </c>
       <c r="D83" s="15" t="n">
-        <v>5800</v>
+        <v>6200</v>
       </c>
       <c r="E83" s="15" t="n">
-        <v>5800</v>
+        <v>6200</v>
       </c>
       <c r="F83" s="15" t="inlineStr">
         <is>
@@ -6033,28 +6033,28 @@
     <row r="84">
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>SOFAB PROVENDERIE</t>
+          <t>KAMGANG EMMANUEL</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>SO2604-52011</t>
+          <t>SO2606-58404</t>
         </is>
       </c>
       <c r="D84" s="15" t="n">
-        <v>4400</v>
+        <v>5800</v>
       </c>
       <c r="E84" s="15" t="n">
-        <v>4400</v>
+        <v>5800</v>
       </c>
       <c r="F84" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G84" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-NDJELENG</t>
         </is>
       </c>
       <c r="H84" s="15" t="inlineStr">
@@ -6071,28 +6071,28 @@
     <row r="85">
       <c r="B85" s="15" t="inlineStr">
         <is>
-          <t>BOUKAR ISAIE</t>
+          <t>SOFAB PROVENDERIE</t>
         </is>
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>SO2604-52017</t>
+          <t>SO2604-52011</t>
         </is>
       </c>
       <c r="D85" s="15" t="n">
-        <v>3100</v>
+        <v>4400</v>
       </c>
       <c r="E85" s="15" t="n">
-        <v>3100</v>
+        <v>4400</v>
       </c>
       <c r="F85" s="15" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G85" s="15" t="inlineStr">
         <is>
-          <t>BELGO-BERI</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H85" s="15" t="inlineStr">
@@ -80629,7 +80629,7 @@
       </c>
       <c r="G6" s="20" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Centre + Littoral</t>
         </is>
       </c>
       <c r="H6" s="20" t="inlineStr"/>

</xml_diff>

<commit_message>
@ v57: TAJOUO 60657 forcee 12 000/12 000 en totalite (ex-10 000) — plan 23/09 = 17 750/15 000 (118%), depassement d eclosion assume (+2 750). 4 forcees, aucune ajoutee par l algo.
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prog poussin/Popo/output/Plan_Livraisons_BELGO_Ponte.xlsx
+++ b/Prog poussin/Popo/output/Plan_Livraisons_BELGO_Ponte.xlsx
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="H7" s="5" t="n">
         <v>12000</v>
@@ -776,7 +776,7 @@
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>LIVRAISON PARTIELLE | Partiel (solde -&gt; production ulterieure) | FORCEE</t>
+          <t>FORCEE</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="6" t="n">
-        <v>15750</v>
+        <v>17750</v>
       </c>
       <c r="G10" s="7" t="n"/>
       <c r="H10" s="7" t="n"/>
@@ -943,7 +943,7 @@
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="8" t="n">
-        <v>15750</v>
+        <v>17750</v>
       </c>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
@@ -1388,7 +1388,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="H7" s="5" t="n">
         <v>12000</v>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>LIVRAISON PARTIELLE | Partiel (solde -&gt; production ulterieure) | FORCEE</t>
+          <t>FORCEE</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="6" t="n">
-        <v>15750</v>
+        <v>17750</v>
       </c>
       <c r="G10" s="7" t="n"/>
       <c r="H10" s="7" t="n"/>
@@ -1592,7 +1592,7 @@
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="8" t="n">
-        <v>15750</v>
+        <v>17750</v>
       </c>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
@@ -1827,7 +1827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I255"/>
+  <dimension ref="B2:I254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8239,19 +8239,19 @@
     <row r="172">
       <c r="B172" s="15" t="inlineStr">
         <is>
-          <t>TAJOUO DAVID</t>
+          <t>KAMADOH MATHIAS</t>
         </is>
       </c>
       <c r="C172" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60657</t>
+          <t>SO2606-60642</t>
         </is>
       </c>
       <c r="D172" s="15" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E172" s="15" t="n">
-        <v>12000</v>
+        <v>1500</v>
       </c>
       <c r="F172" s="15" t="inlineStr">
         <is>
@@ -8277,28 +8277,28 @@
     <row r="173">
       <c r="B173" s="15" t="inlineStr">
         <is>
-          <t>KAMADOH MATHIAS</t>
+          <t>COGESDI SARL</t>
         </is>
       </c>
       <c r="C173" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60642</t>
+          <t>SO2609-69312</t>
         </is>
       </c>
       <c r="D173" s="15" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="E173" s="15" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="F173" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Nord</t>
         </is>
       </c>
       <c r="G173" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-NDERE</t>
         </is>
       </c>
       <c r="H173" s="15" t="inlineStr">
@@ -8308,35 +8308,35 @@
       </c>
       <c r="I173" s="15" t="inlineStr">
         <is>
-          <t>20/11/2026</t>
+          <t>21/11/2026</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="B174" s="15" t="inlineStr">
         <is>
-          <t>COGESDI SARL</t>
+          <t>FIDELIA UCHECK EPSE CHETEU FOMUM</t>
         </is>
       </c>
       <c r="C174" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69312</t>
+          <t>SO2607-62120</t>
         </is>
       </c>
       <c r="D174" s="15" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="E174" s="15" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="F174" s="15" t="inlineStr">
         <is>
-          <t>Nord</t>
+          <t>Est</t>
         </is>
       </c>
       <c r="G174" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDERE</t>
+          <t>BELGO BERTOUA</t>
         </is>
       </c>
       <c r="H174" s="15" t="inlineStr">
@@ -8346,19 +8346,19 @@
       </c>
       <c r="I174" s="15" t="inlineStr">
         <is>
-          <t>21/11/2026</t>
+          <t>22/11/2026</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="B175" s="15" t="inlineStr">
         <is>
-          <t>FIDELIA UCHECK EPSE CHETEU FOMUM</t>
+          <t>COGESDI SARL</t>
         </is>
       </c>
       <c r="C175" s="15" t="inlineStr">
         <is>
-          <t>SO2607-62120</t>
+          <t>SO2609-69306</t>
         </is>
       </c>
       <c r="D175" s="15" t="n">
@@ -8369,12 +8369,12 @@
       </c>
       <c r="F175" s="15" t="inlineStr">
         <is>
-          <t>Est</t>
+          <t>Nord</t>
         </is>
       </c>
       <c r="G175" s="15" t="inlineStr">
         <is>
-          <t>BELGO BERTOUA</t>
+          <t>BELGO-NDERE</t>
         </is>
       </c>
       <c r="H175" s="15" t="inlineStr">
@@ -8391,19 +8391,19 @@
     <row r="176">
       <c r="B176" s="15" t="inlineStr">
         <is>
-          <t>COGESDI SARL</t>
+          <t>HASSAN HAROUNA</t>
         </is>
       </c>
       <c r="C176" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69306</t>
+          <t>SO2609-69136</t>
         </is>
       </c>
       <c r="D176" s="15" t="n">
-        <v>3000</v>
+        <v>1250</v>
       </c>
       <c r="E176" s="15" t="n">
-        <v>3000</v>
+        <v>1250</v>
       </c>
       <c r="F176" s="15" t="inlineStr">
         <is>
@@ -8429,28 +8429,28 @@
     <row r="177">
       <c r="B177" s="15" t="inlineStr">
         <is>
-          <t>HASSAN HAROUNA</t>
+          <t>Kengne Roger</t>
         </is>
       </c>
       <c r="C177" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69136</t>
+          <t>SO2606-59488</t>
         </is>
       </c>
       <c r="D177" s="15" t="n">
-        <v>1250</v>
+        <v>18500</v>
       </c>
       <c r="E177" s="15" t="n">
-        <v>1250</v>
+        <v>18500</v>
       </c>
       <c r="F177" s="15" t="inlineStr">
         <is>
-          <t>Nord</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G177" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDERE</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H177" s="15" t="inlineStr">
@@ -8460,26 +8460,26 @@
       </c>
       <c r="I177" s="15" t="inlineStr">
         <is>
-          <t>22/11/2026</t>
+          <t>25/11/2026</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="B178" s="15" t="inlineStr">
         <is>
-          <t>Kengne Roger</t>
+          <t>NOUTCHOGOUIN TASSE HUBERT</t>
         </is>
       </c>
       <c r="C178" s="15" t="inlineStr">
         <is>
-          <t>SO2606-59488</t>
+          <t>SO2607-61944</t>
         </is>
       </c>
       <c r="D178" s="15" t="n">
-        <v>18500</v>
+        <v>12500</v>
       </c>
       <c r="E178" s="15" t="n">
-        <v>18500</v>
+        <v>12500</v>
       </c>
       <c r="F178" s="15" t="inlineStr">
         <is>
@@ -8505,19 +8505,19 @@
     <row r="179">
       <c r="B179" s="15" t="inlineStr">
         <is>
-          <t>NOUTCHOGOUIN TASSE HUBERT</t>
+          <t>Wokam Kunatse Raymond</t>
         </is>
       </c>
       <c r="C179" s="15" t="inlineStr">
         <is>
-          <t>SO2607-61944</t>
+          <t>SO2607-63052</t>
         </is>
       </c>
       <c r="D179" s="15" t="n">
-        <v>12500</v>
+        <v>3000</v>
       </c>
       <c r="E179" s="15" t="n">
-        <v>12500</v>
+        <v>3000</v>
       </c>
       <c r="F179" s="15" t="inlineStr">
         <is>
@@ -8543,12 +8543,12 @@
     <row r="180">
       <c r="B180" s="15" t="inlineStr">
         <is>
-          <t>Wokam Kunatse Raymond</t>
+          <t>Nganle Alice</t>
         </is>
       </c>
       <c r="C180" s="15" t="inlineStr">
         <is>
-          <t>SO2607-63052</t>
+          <t>SO2607-63390</t>
         </is>
       </c>
       <c r="D180" s="15" t="n">
@@ -8574,35 +8574,35 @@
       </c>
       <c r="I180" s="15" t="inlineStr">
         <is>
-          <t>25/11/2026</t>
+          <t>27/11/2026</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="B181" s="15" t="inlineStr">
         <is>
-          <t>Nganle Alice</t>
+          <t>KAMDOM WATO EPSE MABOU CECILE</t>
         </is>
       </c>
       <c r="C181" s="15" t="inlineStr">
         <is>
-          <t>SO2607-63390</t>
+          <t>SO2608-67154</t>
         </is>
       </c>
       <c r="D181" s="15" t="n">
-        <v>3000</v>
+        <v>50</v>
       </c>
       <c r="E181" s="15" t="n">
-        <v>3000</v>
+        <v>50</v>
       </c>
       <c r="F181" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G181" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H181" s="15" t="inlineStr">
@@ -8612,35 +8612,35 @@
       </c>
       <c r="I181" s="15" t="inlineStr">
         <is>
-          <t>27/11/2026</t>
+          <t>28/11/2026</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="B182" s="15" t="inlineStr">
         <is>
-          <t>KAMDOM WATO EPSE MABOU CECILE</t>
+          <t>Matsing Tené Ange Merveille</t>
         </is>
       </c>
       <c r="C182" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67154</t>
+          <t>SO2606-60455</t>
         </is>
       </c>
       <c r="D182" s="15" t="n">
-        <v>50</v>
+        <v>30000</v>
       </c>
       <c r="E182" s="15" t="n">
-        <v>50</v>
+        <v>30000</v>
       </c>
       <c r="F182" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G182" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-NDJELENG</t>
         </is>
       </c>
       <c r="H182" s="15" t="inlineStr">
@@ -8650,7 +8650,7 @@
       </c>
       <c r="I182" s="15" t="inlineStr">
         <is>
-          <t>28/11/2026</t>
+          <t>04/12/2026</t>
         </is>
       </c>
     </row>
@@ -8662,14 +8662,14 @@
       </c>
       <c r="C183" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60455</t>
+          <t>SO2606-60460</t>
         </is>
       </c>
       <c r="D183" s="15" t="n">
-        <v>30000</v>
+        <v>31000</v>
       </c>
       <c r="E183" s="15" t="n">
-        <v>30000</v>
+        <v>31000</v>
       </c>
       <c r="F183" s="15" t="inlineStr">
         <is>
@@ -8688,26 +8688,26 @@
       </c>
       <c r="I183" s="15" t="inlineStr">
         <is>
-          <t>04/12/2026</t>
+          <t>05/12/2026</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="B184" s="15" t="inlineStr">
         <is>
-          <t>Matsing Tené Ange Merveille</t>
+          <t>FOGANG FOGUM</t>
         </is>
       </c>
       <c r="C184" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60460</t>
+          <t>SO2607-61990</t>
         </is>
       </c>
       <c r="D184" s="15" t="n">
-        <v>31000</v>
+        <v>3200</v>
       </c>
       <c r="E184" s="15" t="n">
-        <v>31000</v>
+        <v>3200</v>
       </c>
       <c r="F184" s="15" t="inlineStr">
         <is>
@@ -8716,7 +8716,7 @@
       </c>
       <c r="G184" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDJELENG</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H184" s="15" t="inlineStr">
@@ -8733,19 +8733,19 @@
     <row r="185">
       <c r="B185" s="15" t="inlineStr">
         <is>
-          <t>FOGANG FOGUM</t>
+          <t>KUE</t>
         </is>
       </c>
       <c r="C185" s="15" t="inlineStr">
         <is>
-          <t>SO2607-61990</t>
+          <t>SO2607-61793</t>
         </is>
       </c>
       <c r="D185" s="15" t="n">
-        <v>3200</v>
+        <v>20050</v>
       </c>
       <c r="E185" s="15" t="n">
-        <v>3200</v>
+        <v>20050</v>
       </c>
       <c r="F185" s="15" t="inlineStr">
         <is>
@@ -8764,35 +8764,35 @@
       </c>
       <c r="I185" s="15" t="inlineStr">
         <is>
-          <t>05/12/2026</t>
+          <t>09/12/2026</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="B186" s="15" t="inlineStr">
         <is>
-          <t>KUE</t>
+          <t>GLORIOUS FARM SARL</t>
         </is>
       </c>
       <c r="C186" s="15" t="inlineStr">
         <is>
-          <t>SO2607-61793</t>
+          <t>SO2606-61535</t>
         </is>
       </c>
       <c r="D186" s="15" t="n">
-        <v>20050</v>
+        <v>17000</v>
       </c>
       <c r="E186" s="15" t="n">
-        <v>20050</v>
+        <v>17000</v>
       </c>
       <c r="F186" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G186" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H186" s="15" t="inlineStr">
@@ -8809,28 +8809,28 @@
     <row r="187">
       <c r="B187" s="15" t="inlineStr">
         <is>
-          <t>GLORIOUS FARM SARL</t>
+          <t>Fotie Tagoumtse Constantin Legrand</t>
         </is>
       </c>
       <c r="C187" s="15" t="inlineStr">
         <is>
-          <t>SO2606-61535</t>
+          <t>SO2607-62146</t>
         </is>
       </c>
       <c r="D187" s="15" t="n">
-        <v>17000</v>
+        <v>5500</v>
       </c>
       <c r="E187" s="15" t="n">
-        <v>17000</v>
+        <v>5500</v>
       </c>
       <c r="F187" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G187" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H187" s="15" t="inlineStr">
@@ -8840,35 +8840,35 @@
       </c>
       <c r="I187" s="15" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>11/12/2026</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="B188" s="15" t="inlineStr">
         <is>
-          <t>Fotie Tagoumtse Constantin Legrand</t>
+          <t>NDIE WILFRED STANLEY</t>
         </is>
       </c>
       <c r="C188" s="15" t="inlineStr">
         <is>
-          <t>SO2607-62146</t>
+          <t>SO2607-61580</t>
         </is>
       </c>
       <c r="D188" s="15" t="n">
-        <v>5500</v>
+        <v>32000</v>
       </c>
       <c r="E188" s="15" t="n">
-        <v>5500</v>
+        <v>32000</v>
       </c>
       <c r="F188" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="G188" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-BERI</t>
         </is>
       </c>
       <c r="H188" s="15" t="inlineStr">
@@ -8878,35 +8878,35 @@
       </c>
       <c r="I188" s="15" t="inlineStr">
         <is>
-          <t>11/12/2026</t>
+          <t>12/12/2026</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="B189" s="15" t="inlineStr">
         <is>
-          <t>NDIE WILFRED STANLEY</t>
+          <t>OUMAROU MAHAMAT</t>
         </is>
       </c>
       <c r="C189" s="15" t="inlineStr">
         <is>
-          <t>SO2607-61580</t>
+          <t>SO2607-65348</t>
         </is>
       </c>
       <c r="D189" s="15" t="n">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="E189" s="15" t="n">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="F189" s="15" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Nord</t>
         </is>
       </c>
       <c r="G189" s="15" t="inlineStr">
         <is>
-          <t>BELGO-BERI</t>
+          <t>BELGO-NDERE</t>
         </is>
       </c>
       <c r="H189" s="15" t="inlineStr">
@@ -8916,35 +8916,35 @@
       </c>
       <c r="I189" s="15" t="inlineStr">
         <is>
-          <t>12/12/2026</t>
+          <t>13/12/2026</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="B190" s="15" t="inlineStr">
         <is>
-          <t>OUMAROU MAHAMAT</t>
+          <t>NDIE WILFRED STANLEY</t>
         </is>
       </c>
       <c r="C190" s="15" t="inlineStr">
         <is>
-          <t>SO2607-65348</t>
+          <t>SO2607-61585</t>
         </is>
       </c>
       <c r="D190" s="15" t="n">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="E190" s="15" t="n">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="F190" s="15" t="inlineStr">
         <is>
-          <t>Nord</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="G190" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDERE</t>
+          <t>BELGO-BERI</t>
         </is>
       </c>
       <c r="H190" s="15" t="inlineStr">
@@ -8954,35 +8954,35 @@
       </c>
       <c r="I190" s="15" t="inlineStr">
         <is>
-          <t>13/12/2026</t>
+          <t>16/12/2026</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="B191" s="15" t="inlineStr">
         <is>
-          <t>NDIE WILFRED STANLEY</t>
+          <t>NOUTCHOGOUI TASSE HUBERT</t>
         </is>
       </c>
       <c r="C191" s="15" t="inlineStr">
         <is>
-          <t>SO2607-61585</t>
+          <t>SO2607-61942</t>
         </is>
       </c>
       <c r="D191" s="15" t="n">
-        <v>13000</v>
+        <v>12500</v>
       </c>
       <c r="E191" s="15" t="n">
-        <v>13000</v>
+        <v>12500</v>
       </c>
       <c r="F191" s="15" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G191" s="15" t="inlineStr">
         <is>
-          <t>BELGO-BERI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H191" s="15" t="inlineStr">
@@ -8999,19 +8999,19 @@
     <row r="192">
       <c r="B192" s="15" t="inlineStr">
         <is>
-          <t>NOUTCHOGOUI TASSE HUBERT</t>
+          <t>KENFACK ALBERT</t>
         </is>
       </c>
       <c r="C192" s="15" t="inlineStr">
         <is>
-          <t>SO2607-61942</t>
+          <t>SO2607-62286</t>
         </is>
       </c>
       <c r="D192" s="15" t="n">
-        <v>12500</v>
+        <v>11000</v>
       </c>
       <c r="E192" s="15" t="n">
-        <v>12500</v>
+        <v>11000</v>
       </c>
       <c r="F192" s="15" t="inlineStr">
         <is>
@@ -9020,7 +9020,7 @@
       </c>
       <c r="G192" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-NDJELENG</t>
         </is>
       </c>
       <c r="H192" s="15" t="inlineStr">
@@ -9037,19 +9037,19 @@
     <row r="193">
       <c r="B193" s="15" t="inlineStr">
         <is>
-          <t>KENFACK ALBERT</t>
+          <t>TAKOULO SAMUEL(GIC REPICO)</t>
         </is>
       </c>
       <c r="C193" s="15" t="inlineStr">
         <is>
-          <t>SO2607-62286</t>
+          <t>SO2609-69263</t>
         </is>
       </c>
       <c r="D193" s="15" t="n">
-        <v>11000</v>
+        <v>1050</v>
       </c>
       <c r="E193" s="15" t="n">
-        <v>11000</v>
+        <v>1050</v>
       </c>
       <c r="F193" s="15" t="inlineStr">
         <is>
@@ -9058,7 +9058,7 @@
       </c>
       <c r="G193" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDJELENG</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H193" s="15" t="inlineStr">
@@ -9075,19 +9075,19 @@
     <row r="194">
       <c r="B194" s="15" t="inlineStr">
         <is>
-          <t>TAKOULO SAMUEL(GIC REPICO)</t>
+          <t>MBOU EPSE TAKADJO ROSINE EBESA</t>
         </is>
       </c>
       <c r="C194" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69263</t>
+          <t>SO2606-60799</t>
         </is>
       </c>
       <c r="D194" s="15" t="n">
-        <v>1050</v>
+        <v>25000</v>
       </c>
       <c r="E194" s="15" t="n">
-        <v>1050</v>
+        <v>25000</v>
       </c>
       <c r="F194" s="15" t="inlineStr">
         <is>
@@ -9096,7 +9096,7 @@
       </c>
       <c r="G194" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-NDJELENG</t>
         </is>
       </c>
       <c r="H194" s="15" t="inlineStr">
@@ -9106,19 +9106,19 @@
       </c>
       <c r="I194" s="15" t="inlineStr">
         <is>
-          <t>16/12/2026</t>
+          <t>18/12/2026</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="B195" s="15" t="inlineStr">
         <is>
-          <t>MBOU EPSE TAKADJO ROSINE EBESA</t>
+          <t>NGNENTEDEM RICHARD</t>
         </is>
       </c>
       <c r="C195" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60799</t>
+          <t>SO2606-60839</t>
         </is>
       </c>
       <c r="D195" s="15" t="n">
@@ -9144,26 +9144,26 @@
       </c>
       <c r="I195" s="15" t="inlineStr">
         <is>
-          <t>18/12/2026</t>
+          <t>19/12/2026</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="B196" s="15" t="inlineStr">
         <is>
-          <t>NGNENTEDEM RICHARD</t>
+          <t>TABOUPDA HENRI</t>
         </is>
       </c>
       <c r="C196" s="15" t="inlineStr">
         <is>
-          <t>SO2606-60839</t>
+          <t>SO2609-68517</t>
         </is>
       </c>
       <c r="D196" s="15" t="n">
-        <v>25000</v>
+        <v>1500</v>
       </c>
       <c r="E196" s="15" t="n">
-        <v>25000</v>
+        <v>1500</v>
       </c>
       <c r="F196" s="15" t="inlineStr">
         <is>
@@ -9172,7 +9172,7 @@
       </c>
       <c r="G196" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDJELENG</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H196" s="15" t="inlineStr">
@@ -9189,19 +9189,19 @@
     <row r="197">
       <c r="B197" s="15" t="inlineStr">
         <is>
-          <t>TABOUPDA HENRI</t>
+          <t>NOUTCHOGOUIN TASSE HUBERT</t>
         </is>
       </c>
       <c r="C197" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68517</t>
+          <t>SO2607-61945</t>
         </is>
       </c>
       <c r="D197" s="15" t="n">
-        <v>1500</v>
+        <v>15000</v>
       </c>
       <c r="E197" s="15" t="n">
-        <v>1500</v>
+        <v>15000</v>
       </c>
       <c r="F197" s="15" t="inlineStr">
         <is>
@@ -9220,26 +9220,26 @@
       </c>
       <c r="I197" s="15" t="inlineStr">
         <is>
-          <t>19/12/2026</t>
+          <t>23/12/2026</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="B198" s="15" t="inlineStr">
         <is>
-          <t>NOUTCHOGOUIN TASSE HUBERT</t>
+          <t>FEUDJIO BACK ARMEL</t>
         </is>
       </c>
       <c r="C198" s="15" t="inlineStr">
         <is>
-          <t>SO2607-61945</t>
+          <t>SO2607-62482</t>
         </is>
       </c>
       <c r="D198" s="15" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E198" s="15" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="F198" s="15" t="inlineStr">
         <is>
@@ -9265,19 +9265,19 @@
     <row r="199">
       <c r="B199" s="15" t="inlineStr">
         <is>
-          <t>FEUDJIO BACK ARMEL</t>
+          <t>TASSE INNOCENT</t>
         </is>
       </c>
       <c r="C199" s="15" t="inlineStr">
         <is>
-          <t>SO2607-62482</t>
+          <t>SO2607-62675</t>
         </is>
       </c>
       <c r="D199" s="15" t="n">
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E199" s="15" t="n">
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="F199" s="15" t="inlineStr">
         <is>
@@ -9303,28 +9303,28 @@
     <row r="200">
       <c r="B200" s="15" t="inlineStr">
         <is>
-          <t>TASSE INNOCENT</t>
+          <t>GIC EMERGENCE</t>
         </is>
       </c>
       <c r="C200" s="15" t="inlineStr">
         <is>
-          <t>SO2607-62675</t>
+          <t>SO2607-64870</t>
         </is>
       </c>
       <c r="D200" s="15" t="n">
-        <v>5700</v>
+        <v>2500</v>
       </c>
       <c r="E200" s="15" t="n">
-        <v>5700</v>
+        <v>2500</v>
       </c>
       <c r="F200" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Est</t>
         </is>
       </c>
       <c r="G200" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO BERTOUA</t>
         </is>
       </c>
       <c r="H200" s="15" t="inlineStr">
@@ -9334,35 +9334,35 @@
       </c>
       <c r="I200" s="15" t="inlineStr">
         <is>
-          <t>23/12/2026</t>
+          <t>24/12/2026</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="B201" s="15" t="inlineStr">
         <is>
-          <t>GIC EMERGENCE</t>
+          <t>FOMEKONG CONSTANT ARNAUD</t>
         </is>
       </c>
       <c r="C201" s="15" t="inlineStr">
         <is>
-          <t>SO2607-64870</t>
+          <t>SO2607-62810</t>
         </is>
       </c>
       <c r="D201" s="15" t="n">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="E201" s="15" t="n">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="F201" s="15" t="inlineStr">
         <is>
-          <t>Est</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G201" s="15" t="inlineStr">
         <is>
-          <t>BELGO BERTOUA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H201" s="15" t="inlineStr">
@@ -9372,35 +9372,35 @@
       </c>
       <c r="I201" s="15" t="inlineStr">
         <is>
-          <t>24/12/2026</t>
+          <t>25/12/2026</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="B202" s="15" t="inlineStr">
         <is>
-          <t>FOMEKONG CONSTANT ARNAUD</t>
+          <t>Nganle Alice</t>
         </is>
       </c>
       <c r="C202" s="15" t="inlineStr">
         <is>
-          <t>SO2607-62810</t>
+          <t>SO2607-63387</t>
         </is>
       </c>
       <c r="D202" s="15" t="n">
-        <v>4000</v>
+        <v>14000</v>
       </c>
       <c r="E202" s="15" t="n">
-        <v>4000</v>
+        <v>14000</v>
       </c>
       <c r="F202" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G202" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H202" s="15" t="inlineStr">
@@ -9410,35 +9410,35 @@
       </c>
       <c r="I202" s="15" t="inlineStr">
         <is>
-          <t>25/12/2026</t>
+          <t>30/12/2026</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="B203" s="15" t="inlineStr">
         <is>
-          <t>Nganle Alice</t>
+          <t>DJOGAM ISIDOR</t>
         </is>
       </c>
       <c r="C203" s="15" t="inlineStr">
         <is>
-          <t>SO2607-63387</t>
+          <t>SO2607-63028</t>
         </is>
       </c>
       <c r="D203" s="15" t="n">
-        <v>14000</v>
+        <v>11000</v>
       </c>
       <c r="E203" s="15" t="n">
-        <v>14000</v>
+        <v>11000</v>
       </c>
       <c r="F203" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G203" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H203" s="15" t="inlineStr">
@@ -9455,28 +9455,28 @@
     <row r="204">
       <c r="B204" s="15" t="inlineStr">
         <is>
-          <t>DJOGAM ISIDOR</t>
+          <t>KUEDAHA TEDONGMO MARIUS</t>
         </is>
       </c>
       <c r="C204" s="15" t="inlineStr">
         <is>
-          <t>SO2607-63028</t>
+          <t>SO2606-58943</t>
         </is>
       </c>
       <c r="D204" s="15" t="n">
-        <v>11000</v>
+        <v>5200</v>
       </c>
       <c r="E204" s="15" t="n">
-        <v>11000</v>
+        <v>5200</v>
       </c>
       <c r="F204" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G204" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-NDJELENG</t>
         </is>
       </c>
       <c r="H204" s="15" t="inlineStr">
@@ -9493,28 +9493,28 @@
     <row r="205">
       <c r="B205" s="15" t="inlineStr">
         <is>
-          <t>KUEDAHA TEDONGMO MARIUS</t>
+          <t>KUHLIFARM COOP-BOD (KUMBA KOPEFUL LIVESTOCK FARMERS)</t>
         </is>
       </c>
       <c r="C205" s="15" t="inlineStr">
         <is>
-          <t>SO2606-58943</t>
+          <t>SO2607-64720</t>
         </is>
       </c>
       <c r="D205" s="15" t="n">
-        <v>5200</v>
+        <v>5000</v>
       </c>
       <c r="E205" s="15" t="n">
-        <v>5200</v>
+        <v>5000</v>
       </c>
       <c r="F205" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="G205" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDJELENG</t>
+          <t>BELGO-BERI</t>
         </is>
       </c>
       <c r="H205" s="15" t="inlineStr">
@@ -9531,28 +9531,28 @@
     <row r="206">
       <c r="B206" s="15" t="inlineStr">
         <is>
-          <t>KUHLIFARM COOP-BOD (KUMBA KOPEFUL LIVESTOCK FARMERS)</t>
+          <t>GIC DES AGRICULTEURS DE TSINGBEU</t>
         </is>
       </c>
       <c r="C206" s="15" t="inlineStr">
         <is>
-          <t>SO2607-64720</t>
+          <t>SO2608-66811</t>
         </is>
       </c>
       <c r="D206" s="15" t="n">
-        <v>5000</v>
+        <v>22000</v>
       </c>
       <c r="E206" s="15" t="n">
-        <v>5000</v>
+        <v>22000</v>
       </c>
       <c r="F206" s="15" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G206" s="15" t="inlineStr">
         <is>
-          <t>BELGO-BERI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H206" s="15" t="inlineStr">
@@ -9562,26 +9562,26 @@
       </c>
       <c r="I206" s="15" t="inlineStr">
         <is>
-          <t>30/12/2026</t>
+          <t>06/01/2027</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="B207" s="15" t="inlineStr">
         <is>
-          <t>GIC DES AGRICULTEURS DE TSINGBEU</t>
+          <t>TCHIFFO</t>
         </is>
       </c>
       <c r="C207" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66811</t>
+          <t>SO2608-67018</t>
         </is>
       </c>
       <c r="D207" s="15" t="n">
-        <v>22000</v>
+        <v>5200</v>
       </c>
       <c r="E207" s="15" t="n">
-        <v>22000</v>
+        <v>5200</v>
       </c>
       <c r="F207" s="15" t="inlineStr">
         <is>
@@ -9612,14 +9612,14 @@
       </c>
       <c r="C208" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67018</t>
+          <t>SO2608-67017</t>
         </is>
       </c>
       <c r="D208" s="15" t="n">
-        <v>5200</v>
+        <v>2000</v>
       </c>
       <c r="E208" s="15" t="n">
-        <v>5200</v>
+        <v>2000</v>
       </c>
       <c r="F208" s="15" t="inlineStr">
         <is>
@@ -9645,28 +9645,28 @@
     <row r="209">
       <c r="B209" s="15" t="inlineStr">
         <is>
-          <t>TCHIFFO</t>
+          <t>RAYMOND MINKULA NGOE (MINKO MANAGEMENT AND LOGISTIC SCES)</t>
         </is>
       </c>
       <c r="C209" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67017</t>
+          <t>SO2608-66839</t>
         </is>
       </c>
       <c r="D209" s="15" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E209" s="15" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="F209" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="G209" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-BERI</t>
         </is>
       </c>
       <c r="H209" s="15" t="inlineStr">
@@ -9683,28 +9683,28 @@
     <row r="210">
       <c r="B210" s="15" t="inlineStr">
         <is>
-          <t>RAYMOND MINKULA NGOE (MINKO MANAGEMENT AND LOGISTIC SCES)</t>
+          <t>KAMGANG SIMPLICE</t>
         </is>
       </c>
       <c r="C210" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66839</t>
+          <t>SO2608-66886</t>
         </is>
       </c>
       <c r="D210" s="15" t="n">
-        <v>1500</v>
+        <v>30700</v>
       </c>
       <c r="E210" s="15" t="n">
-        <v>1500</v>
+        <v>30700</v>
       </c>
       <c r="F210" s="15" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G210" s="15" t="inlineStr">
         <is>
-          <t>BELGO-BERI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H210" s="15" t="inlineStr">
@@ -9714,35 +9714,35 @@
       </c>
       <c r="I210" s="15" t="inlineStr">
         <is>
-          <t>06/01/2027</t>
+          <t>07/01/2027</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="B211" s="15" t="inlineStr">
         <is>
-          <t>KAMGANG SIMPLICE</t>
+          <t>GIC PATBEN FARM (SISHU YESINVEM NESTOR)</t>
         </is>
       </c>
       <c r="C211" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66886</t>
+          <t>SO2609-68925</t>
         </is>
       </c>
       <c r="D211" s="15" t="n">
-        <v>30700</v>
+        <v>16000</v>
       </c>
       <c r="E211" s="15" t="n">
-        <v>30700</v>
+        <v>16000</v>
       </c>
       <c r="F211" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G211" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H211" s="15" t="inlineStr">
@@ -9759,28 +9759,28 @@
     <row r="212">
       <c r="B212" s="15" t="inlineStr">
         <is>
-          <t>GIC PATBEN FARM (SISHU YESINVEM NESTOR)</t>
+          <t>WAN POULTRY</t>
         </is>
       </c>
       <c r="C212" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68925</t>
+          <t>SO2609-68938</t>
         </is>
       </c>
       <c r="D212" s="15" t="n">
-        <v>16000</v>
+        <v>5000</v>
       </c>
       <c r="E212" s="15" t="n">
-        <v>16000</v>
+        <v>5000</v>
       </c>
       <c r="F212" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G212" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO MBOUDA</t>
         </is>
       </c>
       <c r="H212" s="15" t="inlineStr">
@@ -9797,19 +9797,19 @@
     <row r="213">
       <c r="B213" s="15" t="inlineStr">
         <is>
-          <t>WAN POULTRY</t>
+          <t>KAMGANG SIMPLICE</t>
         </is>
       </c>
       <c r="C213" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68938</t>
+          <t>SO2608-66888</t>
         </is>
       </c>
       <c r="D213" s="15" t="n">
-        <v>5000</v>
+        <v>30700</v>
       </c>
       <c r="E213" s="15" t="n">
-        <v>5000</v>
+        <v>30700</v>
       </c>
       <c r="F213" s="15" t="inlineStr">
         <is>
@@ -9818,7 +9818,7 @@
       </c>
       <c r="G213" s="15" t="inlineStr">
         <is>
-          <t>BELGO MBOUDA</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H213" s="15" t="inlineStr">
@@ -9828,35 +9828,35 @@
       </c>
       <c r="I213" s="15" t="inlineStr">
         <is>
-          <t>07/01/2027</t>
+          <t>09/01/2027</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="B214" s="15" t="inlineStr">
         <is>
-          <t>KAMGANG SIMPLICE</t>
+          <t>SOFAB PROVENDERIE</t>
         </is>
       </c>
       <c r="C214" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66888</t>
+          <t>SO2609-69180</t>
         </is>
       </c>
       <c r="D214" s="15" t="n">
-        <v>30700</v>
+        <v>8000</v>
       </c>
       <c r="E214" s="15" t="n">
-        <v>30700</v>
+        <v>8000</v>
       </c>
       <c r="F214" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G214" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H214" s="15" t="inlineStr">
@@ -9873,19 +9873,19 @@
     <row r="215">
       <c r="B215" s="15" t="inlineStr">
         <is>
-          <t>SOFAB PROVENDERIE</t>
+          <t>PROVENDERIE L'EMERGENCE (SIAGA SIANI MARTIAL)</t>
         </is>
       </c>
       <c r="C215" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69180</t>
+          <t>SO2609-69033</t>
         </is>
       </c>
       <c r="D215" s="15" t="n">
-        <v>8000</v>
+        <v>4500</v>
       </c>
       <c r="E215" s="15" t="n">
-        <v>8000</v>
+        <v>4500</v>
       </c>
       <c r="F215" s="15" t="inlineStr">
         <is>
@@ -9894,7 +9894,7 @@
       </c>
       <c r="G215" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO AHALA</t>
         </is>
       </c>
       <c r="H215" s="15" t="inlineStr">
@@ -9911,28 +9911,28 @@
     <row r="216">
       <c r="B216" s="15" t="inlineStr">
         <is>
-          <t>PROVENDERIE L'EMERGENCE (SIAGA SIANI MARTIAL)</t>
+          <t>KAMGANG SIMPLICE</t>
         </is>
       </c>
       <c r="C216" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69033</t>
+          <t>SO2608-66889</t>
         </is>
       </c>
       <c r="D216" s="15" t="n">
-        <v>4500</v>
+        <v>8600</v>
       </c>
       <c r="E216" s="15" t="n">
-        <v>4500</v>
+        <v>8600</v>
       </c>
       <c r="F216" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G216" s="15" t="inlineStr">
         <is>
-          <t>BELGO AHALA</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H216" s="15" t="inlineStr">
@@ -9942,35 +9942,35 @@
       </c>
       <c r="I216" s="15" t="inlineStr">
         <is>
-          <t>09/01/2027</t>
+          <t>12/01/2027</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="B217" s="15" t="inlineStr">
         <is>
-          <t>KAMGANG SIMPLICE</t>
+          <t>FOFOU SIMPHORIN</t>
         </is>
       </c>
       <c r="C217" s="15" t="inlineStr">
         <is>
-          <t>SO2608-66889</t>
+          <t>SO2608-67028</t>
         </is>
       </c>
       <c r="D217" s="15" t="n">
-        <v>8600</v>
+        <v>8000</v>
       </c>
       <c r="E217" s="15" t="n">
-        <v>8600</v>
+        <v>8000</v>
       </c>
       <c r="F217" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G217" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H217" s="15" t="inlineStr">
@@ -9987,19 +9987,19 @@
     <row r="218">
       <c r="B218" s="15" t="inlineStr">
         <is>
-          <t>FOFOU SIMPHORIN</t>
+          <t>BOGNING</t>
         </is>
       </c>
       <c r="C218" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67028</t>
+          <t>SO2608-67035</t>
         </is>
       </c>
       <c r="D218" s="15" t="n">
-        <v>8000</v>
+        <v>5000</v>
       </c>
       <c r="E218" s="15" t="n">
-        <v>8000</v>
+        <v>5000</v>
       </c>
       <c r="F218" s="15" t="inlineStr">
         <is>
@@ -10025,19 +10025,19 @@
     <row r="219">
       <c r="B219" s="15" t="inlineStr">
         <is>
-          <t>BOGNING</t>
+          <t>Societe Agro Pastorale ( Sap)</t>
         </is>
       </c>
       <c r="C219" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67035</t>
+          <t>SO2609-69188</t>
         </is>
       </c>
       <c r="D219" s="15" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="E219" s="15" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="F219" s="15" t="inlineStr">
         <is>
@@ -10063,19 +10063,19 @@
     <row r="220">
       <c r="B220" s="15" t="inlineStr">
         <is>
-          <t>Societe Agro Pastorale ( Sap)</t>
+          <t>DANG CHRISTIAN (DANG CHRISTIAN)</t>
         </is>
       </c>
       <c r="C220" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69188</t>
+          <t>SO2609-68964</t>
         </is>
       </c>
       <c r="D220" s="15" t="n">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="E220" s="15" t="n">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="F220" s="15" t="inlineStr">
         <is>
@@ -10084,7 +10084,7 @@
       </c>
       <c r="G220" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO AHALA</t>
         </is>
       </c>
       <c r="H220" s="15" t="inlineStr">
@@ -10101,28 +10101,28 @@
     <row r="221">
       <c r="B221" s="15" t="inlineStr">
         <is>
-          <t>DANG CHRISTIAN (DANG CHRISTIAN)</t>
+          <t>TCHIFFO</t>
         </is>
       </c>
       <c r="C221" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68964</t>
+          <t>SO2608-67016</t>
         </is>
       </c>
       <c r="D221" s="15" t="n">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="E221" s="15" t="n">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="F221" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G221" s="15" t="inlineStr">
         <is>
-          <t>BELGO AHALA</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H221" s="15" t="inlineStr">
@@ -10132,26 +10132,26 @@
       </c>
       <c r="I221" s="15" t="inlineStr">
         <is>
-          <t>12/01/2027</t>
+          <t>13/01/2027</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="B222" s="15" t="inlineStr">
         <is>
-          <t>TCHIFFO</t>
+          <t>Tchinda Kuekou Victor</t>
         </is>
       </c>
       <c r="C222" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67016</t>
+          <t>SO2608-67060</t>
         </is>
       </c>
       <c r="D222" s="15" t="n">
-        <v>30000</v>
+        <v>9000</v>
       </c>
       <c r="E222" s="15" t="n">
-        <v>30000</v>
+        <v>9000</v>
       </c>
       <c r="F222" s="15" t="inlineStr">
         <is>
@@ -10170,35 +10170,35 @@
       </c>
       <c r="I222" s="15" t="inlineStr">
         <is>
-          <t>13/01/2027</t>
+          <t>15/01/2027</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="B223" s="15" t="inlineStr">
         <is>
-          <t>Tchinda Kuekou Victor</t>
+          <t>FOFOU SIMPHORIN</t>
         </is>
       </c>
       <c r="C223" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67060</t>
+          <t>SO2608-67136</t>
         </is>
       </c>
       <c r="D223" s="15" t="n">
-        <v>9000</v>
+        <v>7150</v>
       </c>
       <c r="E223" s="15" t="n">
-        <v>9000</v>
+        <v>7150</v>
       </c>
       <c r="F223" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G223" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H223" s="15" t="inlineStr">
@@ -10215,28 +10215,28 @@
     <row r="224">
       <c r="B224" s="15" t="inlineStr">
         <is>
-          <t>FOFOU SIMPHORIN</t>
+          <t>Dzudjo Emmanuel</t>
         </is>
       </c>
       <c r="C224" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67136</t>
+          <t>SO2608-67052</t>
         </is>
       </c>
       <c r="D224" s="15" t="n">
-        <v>7150</v>
+        <v>5000</v>
       </c>
       <c r="E224" s="15" t="n">
-        <v>7150</v>
+        <v>5000</v>
       </c>
       <c r="F224" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G224" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H224" s="15" t="inlineStr">
@@ -10253,19 +10253,19 @@
     <row r="225">
       <c r="B225" s="15" t="inlineStr">
         <is>
-          <t>Dzudjo Emmanuel</t>
+          <t>KUATE FRANKY</t>
         </is>
       </c>
       <c r="C225" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67052</t>
+          <t>SO2608-68286</t>
         </is>
       </c>
       <c r="D225" s="15" t="n">
-        <v>5000</v>
+        <v>850</v>
       </c>
       <c r="E225" s="15" t="n">
-        <v>5000</v>
+        <v>850</v>
       </c>
       <c r="F225" s="15" t="inlineStr">
         <is>
@@ -10284,35 +10284,35 @@
       </c>
       <c r="I225" s="15" t="inlineStr">
         <is>
-          <t>15/01/2027</t>
+          <t>19/01/2027</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="B226" s="15" t="inlineStr">
         <is>
-          <t>KUATE FRANKY</t>
+          <t>Maleudjou Kom Epse Tamto Dorisse Michaelle</t>
         </is>
       </c>
       <c r="C226" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68286</t>
+          <t>SO2608-67277</t>
         </is>
       </c>
       <c r="D226" s="15" t="n">
-        <v>850</v>
+        <v>3300</v>
       </c>
       <c r="E226" s="15" t="n">
-        <v>850</v>
+        <v>3300</v>
       </c>
       <c r="F226" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="G226" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-NKONGSAMBA</t>
         </is>
       </c>
       <c r="H226" s="15" t="inlineStr">
@@ -10329,19 +10329,19 @@
     <row r="227">
       <c r="B227" s="15" t="inlineStr">
         <is>
-          <t>Maleudjou Kom Epse Tamto Dorisse Michaelle</t>
+          <t>VOKENG KENANG GUILIANO HERVE</t>
         </is>
       </c>
       <c r="C227" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67277</t>
+          <t>SO2608-67313</t>
         </is>
       </c>
       <c r="D227" s="15" t="n">
-        <v>3300</v>
+        <v>2200</v>
       </c>
       <c r="E227" s="15" t="n">
-        <v>3300</v>
+        <v>2200</v>
       </c>
       <c r="F227" s="15" t="inlineStr">
         <is>
@@ -10350,7 +10350,7 @@
       </c>
       <c r="G227" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NKONGSAMBA</t>
+          <t>BELGO-BERI</t>
         </is>
       </c>
       <c r="H227" s="15" t="inlineStr">
@@ -10367,28 +10367,28 @@
     <row r="228">
       <c r="B228" s="15" t="inlineStr">
         <is>
-          <t>VOKENG KENANG GUILIANO HERVE</t>
+          <t>FOKA TAPOK LAURENT FABRICE</t>
         </is>
       </c>
       <c r="C228" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67313</t>
+          <t>SO2608-67251</t>
         </is>
       </c>
       <c r="D228" s="15" t="n">
-        <v>2200</v>
+        <v>2000</v>
       </c>
       <c r="E228" s="15" t="n">
-        <v>2200</v>
+        <v>2000</v>
       </c>
       <c r="F228" s="15" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G228" s="15" t="inlineStr">
         <is>
-          <t>BELGO-BERI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H228" s="15" t="inlineStr">
@@ -10405,28 +10405,28 @@
     <row r="229">
       <c r="B229" s="15" t="inlineStr">
         <is>
-          <t>FOKA TAPOK LAURENT FABRICE</t>
+          <t>SOFAB PROVENDERIE</t>
         </is>
       </c>
       <c r="C229" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67251</t>
+          <t>SO2609-69231</t>
         </is>
       </c>
       <c r="D229" s="15" t="n">
-        <v>2000</v>
+        <v>5500</v>
       </c>
       <c r="E229" s="15" t="n">
-        <v>2000</v>
+        <v>5500</v>
       </c>
       <c r="F229" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G229" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H229" s="15" t="inlineStr">
@@ -10436,35 +10436,35 @@
       </c>
       <c r="I229" s="15" t="inlineStr">
         <is>
-          <t>19/01/2027</t>
+          <t>20/01/2027</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="B230" s="15" t="inlineStr">
         <is>
-          <t>SOFAB PROVENDERIE</t>
+          <t>GIC AMOUR</t>
         </is>
       </c>
       <c r="C230" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69231</t>
+          <t>SO2608-67259</t>
         </is>
       </c>
       <c r="D230" s="15" t="n">
-        <v>5500</v>
+        <v>10500</v>
       </c>
       <c r="E230" s="15" t="n">
-        <v>5500</v>
+        <v>10500</v>
       </c>
       <c r="F230" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G230" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H230" s="15" t="inlineStr">
@@ -10474,26 +10474,26 @@
       </c>
       <c r="I230" s="15" t="inlineStr">
         <is>
-          <t>20/01/2027</t>
+          <t>22/01/2027</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="B231" s="15" t="inlineStr">
         <is>
-          <t>GIC AMOUR</t>
+          <t>NJOUNDIYIMOUN PAUL DESIRE</t>
         </is>
       </c>
       <c r="C231" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67259</t>
+          <t>SO2608-67500</t>
         </is>
       </c>
       <c r="D231" s="15" t="n">
-        <v>10500</v>
+        <v>2200</v>
       </c>
       <c r="E231" s="15" t="n">
-        <v>10500</v>
+        <v>2200</v>
       </c>
       <c r="F231" s="15" t="inlineStr">
         <is>
@@ -10519,28 +10519,28 @@
     <row r="232">
       <c r="B232" s="15" t="inlineStr">
         <is>
-          <t>NJOUNDIYIMOUN PAUL DESIRE</t>
+          <t>TALOM TELESPHORE</t>
         </is>
       </c>
       <c r="C232" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67500</t>
+          <t>SO2608-67540</t>
         </is>
       </c>
       <c r="D232" s="15" t="n">
-        <v>2200</v>
+        <v>2100</v>
       </c>
       <c r="E232" s="15" t="n">
-        <v>2200</v>
+        <v>2100</v>
       </c>
       <c r="F232" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G232" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H232" s="15" t="inlineStr">
@@ -10557,28 +10557,28 @@
     <row r="233">
       <c r="B233" s="15" t="inlineStr">
         <is>
-          <t>TALOM TELESPHORE</t>
+          <t>TAKETCHOUOP TIWE JUSTIN</t>
         </is>
       </c>
       <c r="C233" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67540</t>
+          <t>SO2608-68078</t>
         </is>
       </c>
       <c r="D233" s="15" t="n">
-        <v>2100</v>
+        <v>1500</v>
       </c>
       <c r="E233" s="15" t="n">
-        <v>2100</v>
+        <v>1500</v>
       </c>
       <c r="F233" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G233" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H233" s="15" t="inlineStr">
@@ -10595,28 +10595,28 @@
     <row r="234">
       <c r="B234" s="15" t="inlineStr">
         <is>
-          <t>TAKETCHOUOP TIWE JUSTIN</t>
+          <t>TD EMERGENCE SARL (TALOM GUENO DIEUDONNE)</t>
         </is>
       </c>
       <c r="C234" s="15" t="inlineStr">
         <is>
-          <t>SO2608-68078</t>
+          <t>SO2608-67410</t>
         </is>
       </c>
       <c r="D234" s="15" t="n">
-        <v>1500</v>
+        <v>1100</v>
       </c>
       <c r="E234" s="15" t="n">
-        <v>1500</v>
+        <v>1100</v>
       </c>
       <c r="F234" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G234" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO AHALA</t>
         </is>
       </c>
       <c r="H234" s="15" t="inlineStr">
@@ -10633,19 +10633,19 @@
     <row r="235">
       <c r="B235" s="15" t="inlineStr">
         <is>
-          <t>TD EMERGENCE SARL (TALOM GUENO DIEUDONNE)</t>
+          <t>TALOM TELESPHORE</t>
         </is>
       </c>
       <c r="C235" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67410</t>
+          <t>SO2608-67443</t>
         </is>
       </c>
       <c r="D235" s="15" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E235" s="15" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="F235" s="15" t="inlineStr">
         <is>
@@ -10654,7 +10654,7 @@
       </c>
       <c r="G235" s="15" t="inlineStr">
         <is>
-          <t>BELGO AHALA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H235" s="15" t="inlineStr">
@@ -10671,28 +10671,28 @@
     <row r="236">
       <c r="B236" s="15" t="inlineStr">
         <is>
-          <t>TALOM TELESPHORE</t>
+          <t>FOTSA FERDINAND</t>
         </is>
       </c>
       <c r="C236" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67443</t>
+          <t>SO2608-67766</t>
         </is>
       </c>
       <c r="D236" s="15" t="n">
-        <v>1050</v>
+        <v>900</v>
       </c>
       <c r="E236" s="15" t="n">
-        <v>1050</v>
+        <v>900</v>
       </c>
       <c r="F236" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G236" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-NDJELENG</t>
         </is>
       </c>
       <c r="H236" s="15" t="inlineStr">
@@ -10702,35 +10702,35 @@
       </c>
       <c r="I236" s="15" t="inlineStr">
         <is>
-          <t>22/01/2027</t>
+          <t>26/01/2027</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="B237" s="15" t="inlineStr">
         <is>
-          <t>FOTSA FERDINAND</t>
+          <t>KAMDEM MERLIN</t>
         </is>
       </c>
       <c r="C237" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67766</t>
+          <t>SO2608-67552</t>
         </is>
       </c>
       <c r="D237" s="15" t="n">
-        <v>900</v>
+        <v>11000</v>
       </c>
       <c r="E237" s="15" t="n">
-        <v>900</v>
+        <v>11000</v>
       </c>
       <c r="F237" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G237" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NDJELENG</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H237" s="15" t="inlineStr">
@@ -10747,28 +10747,28 @@
     <row r="238">
       <c r="B238" s="15" t="inlineStr">
         <is>
-          <t>KAMDEM MERLIN</t>
+          <t>TAMOU JEAN ROBERT</t>
         </is>
       </c>
       <c r="C238" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67552</t>
+          <t>SO2608-67538</t>
         </is>
       </c>
       <c r="D238" s="15" t="n">
-        <v>11000</v>
+        <v>6300</v>
       </c>
       <c r="E238" s="15" t="n">
-        <v>11000</v>
+        <v>6300</v>
       </c>
       <c r="F238" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G238" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H238" s="15" t="inlineStr">
@@ -10785,19 +10785,19 @@
     <row r="239">
       <c r="B239" s="15" t="inlineStr">
         <is>
-          <t>TAMOU JEAN ROBERT</t>
+          <t>KUEGHANG RIGOBERT</t>
         </is>
       </c>
       <c r="C239" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67538</t>
+          <t>SO2609-69215</t>
         </is>
       </c>
       <c r="D239" s="15" t="n">
-        <v>6300</v>
+        <v>10850</v>
       </c>
       <c r="E239" s="15" t="n">
-        <v>6300</v>
+        <v>10850</v>
       </c>
       <c r="F239" s="15" t="inlineStr">
         <is>
@@ -10816,26 +10816,26 @@
       </c>
       <c r="I239" s="15" t="inlineStr">
         <is>
-          <t>26/01/2027</t>
+          <t>27/01/2027</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="B240" s="15" t="inlineStr">
         <is>
-          <t>KUEGHANG RIGOBERT</t>
+          <t>TAMOU JEAN ROBERT</t>
         </is>
       </c>
       <c r="C240" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69215</t>
+          <t>SO2609-69138</t>
         </is>
       </c>
       <c r="D240" s="15" t="n">
-        <v>10850</v>
+        <v>10000</v>
       </c>
       <c r="E240" s="15" t="n">
-        <v>10850</v>
+        <v>10000</v>
       </c>
       <c r="F240" s="15" t="inlineStr">
         <is>
@@ -10861,28 +10861,28 @@
     <row r="241">
       <c r="B241" s="15" t="inlineStr">
         <is>
-          <t>TAMOU JEAN ROBERT</t>
+          <t>Menanpo Nono Nadia</t>
         </is>
       </c>
       <c r="C241" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69138</t>
+          <t>SO2609-69232</t>
         </is>
       </c>
       <c r="D241" s="15" t="n">
-        <v>10000</v>
+        <v>4500</v>
       </c>
       <c r="E241" s="15" t="n">
-        <v>10000</v>
+        <v>4500</v>
       </c>
       <c r="F241" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G241" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H241" s="15" t="inlineStr">
@@ -10899,19 +10899,19 @@
     <row r="242">
       <c r="B242" s="15" t="inlineStr">
         <is>
-          <t>Menanpo Nono Nadia</t>
+          <t>CHIMINYI AWUDOU PANGTAMPEH</t>
         </is>
       </c>
       <c r="C242" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69232</t>
+          <t>SO2609-69543</t>
         </is>
       </c>
       <c r="D242" s="15" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="E242" s="15" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="F242" s="15" t="inlineStr">
         <is>
@@ -10920,7 +10920,7 @@
       </c>
       <c r="G242" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-NKOLBISSON</t>
         </is>
       </c>
       <c r="H242" s="15" t="inlineStr">
@@ -10937,19 +10937,19 @@
     <row r="243">
       <c r="B243" s="15" t="inlineStr">
         <is>
-          <t>CHIMINYI AWUDOU PANGTAMPEH</t>
+          <t>KAMDEM MERLIN</t>
         </is>
       </c>
       <c r="C243" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69543</t>
+          <t>SO2608-67550</t>
         </is>
       </c>
       <c r="D243" s="15" t="n">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="E243" s="15" t="n">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="F243" s="15" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="G243" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NKOLBISSON</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H243" s="15" t="inlineStr">
@@ -10968,35 +10968,35 @@
       </c>
       <c r="I243" s="15" t="inlineStr">
         <is>
-          <t>27/01/2027</t>
+          <t>29/01/2027</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="B244" s="15" t="inlineStr">
         <is>
-          <t>KAMDEM MERLIN</t>
+          <t>TEIKING JEAN MARIE</t>
         </is>
       </c>
       <c r="C244" s="15" t="inlineStr">
         <is>
-          <t>SO2608-67550</t>
+          <t>SO2609-69409</t>
         </is>
       </c>
       <c r="D244" s="15" t="n">
-        <v>30000</v>
+        <v>26000</v>
       </c>
       <c r="E244" s="15" t="n">
-        <v>30000</v>
+        <v>26000</v>
       </c>
       <c r="F244" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G244" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H244" s="15" t="inlineStr">
@@ -11006,35 +11006,35 @@
       </c>
       <c r="I244" s="15" t="inlineStr">
         <is>
-          <t>29/01/2027</t>
+          <t>02/02/2027</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="B245" s="15" t="inlineStr">
         <is>
-          <t>TEIKING JEAN MARIE</t>
+          <t>KOM BLAISE Mr</t>
         </is>
       </c>
       <c r="C245" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69409</t>
+          <t>SO2609-69643</t>
         </is>
       </c>
       <c r="D245" s="15" t="n">
-        <v>26000</v>
+        <v>10200</v>
       </c>
       <c r="E245" s="15" t="n">
-        <v>26000</v>
+        <v>10200</v>
       </c>
       <c r="F245" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G245" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H245" s="15" t="inlineStr">
@@ -11044,35 +11044,35 @@
       </c>
       <c r="I245" s="15" t="inlineStr">
         <is>
-          <t>02/02/2027</t>
+          <t>05/02/2027</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="B246" s="15" t="inlineStr">
         <is>
-          <t>KOM BLAISE Mr</t>
+          <t>IBII OTTO</t>
         </is>
       </c>
       <c r="C246" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69643</t>
+          <t>SO2609-69640</t>
         </is>
       </c>
       <c r="D246" s="15" t="n">
-        <v>10200</v>
+        <v>10150</v>
       </c>
       <c r="E246" s="15" t="n">
-        <v>10200</v>
+        <v>10150</v>
       </c>
       <c r="F246" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="G246" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO PK11</t>
         </is>
       </c>
       <c r="H246" s="15" t="inlineStr">
@@ -11089,28 +11089,28 @@
     <row r="247">
       <c r="B247" s="15" t="inlineStr">
         <is>
-          <t>IBII OTTO</t>
+          <t>SOFAB PROVENDERIE</t>
         </is>
       </c>
       <c r="C247" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69640</t>
+          <t>SO2609-69320</t>
         </is>
       </c>
       <c r="D247" s="15" t="n">
-        <v>10150</v>
+        <v>4200</v>
       </c>
       <c r="E247" s="15" t="n">
-        <v>10150</v>
+        <v>4200</v>
       </c>
       <c r="F247" s="15" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G247" s="15" t="inlineStr">
         <is>
-          <t>BELGO PK11</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H247" s="15" t="inlineStr">
@@ -11127,19 +11127,19 @@
     <row r="248">
       <c r="B248" s="15" t="inlineStr">
         <is>
-          <t>SOFAB PROVENDERIE</t>
+          <t>MODZE WAMBO EPSE TIANTSE</t>
         </is>
       </c>
       <c r="C248" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69320</t>
+          <t>SO2609-69594</t>
         </is>
       </c>
       <c r="D248" s="15" t="n">
-        <v>4200</v>
+        <v>6600</v>
       </c>
       <c r="E248" s="15" t="n">
-        <v>4200</v>
+        <v>6600</v>
       </c>
       <c r="F248" s="15" t="inlineStr">
         <is>
@@ -11158,35 +11158,35 @@
       </c>
       <c r="I248" s="15" t="inlineStr">
         <is>
-          <t>05/02/2027</t>
+          <t>09/02/2027</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="B249" s="15" t="inlineStr">
         <is>
-          <t>MODZE WAMBO EPSE TIANTSE</t>
+          <t>NGOUMDOUM AUGUSTIN</t>
         </is>
       </c>
       <c r="C249" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69594</t>
+          <t>SO2609-69813</t>
         </is>
       </c>
       <c r="D249" s="15" t="n">
-        <v>6600</v>
+        <v>23000</v>
       </c>
       <c r="E249" s="15" t="n">
-        <v>6600</v>
+        <v>23000</v>
       </c>
       <c r="F249" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G249" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H249" s="15" t="inlineStr">
@@ -11196,26 +11196,26 @@
       </c>
       <c r="I249" s="15" t="inlineStr">
         <is>
-          <t>09/02/2027</t>
+          <t>10/02/2027</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="B250" s="15" t="inlineStr">
         <is>
-          <t>NGOUMDOUM AUGUSTIN</t>
+          <t>SAGUEN DEFFO JEAN</t>
         </is>
       </c>
       <c r="C250" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69813</t>
+          <t>SO2609-69831</t>
         </is>
       </c>
       <c r="D250" s="15" t="n">
-        <v>23000</v>
+        <v>25000</v>
       </c>
       <c r="E250" s="15" t="n">
-        <v>23000</v>
+        <v>25000</v>
       </c>
       <c r="F250" s="15" t="inlineStr">
         <is>
@@ -11234,35 +11234,35 @@
       </c>
       <c r="I250" s="15" t="inlineStr">
         <is>
-          <t>10/02/2027</t>
+          <t>12/02/2027</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="B251" s="15" t="inlineStr">
         <is>
-          <t>SAGUEN DEFFO JEAN</t>
+          <t>Kealack Fidele</t>
         </is>
       </c>
       <c r="C251" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69831</t>
+          <t>SO2609-69603</t>
         </is>
       </c>
       <c r="D251" s="15" t="n">
-        <v>25000</v>
+        <v>5100</v>
       </c>
       <c r="E251" s="15" t="n">
-        <v>25000</v>
+        <v>5100</v>
       </c>
       <c r="F251" s="15" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G251" s="15" t="inlineStr">
         <is>
-          <t>BELGO-FAMLA</t>
+          <t>BELGO-MESSASSI</t>
         </is>
       </c>
       <c r="H251" s="15" t="inlineStr">
@@ -11272,26 +11272,26 @@
       </c>
       <c r="I251" s="15" t="inlineStr">
         <is>
-          <t>12/02/2027</t>
+          <t>16/02/2027</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="B252" s="15" t="inlineStr">
         <is>
-          <t>Kealack Fidele</t>
+          <t>GLOBAL BUSINESS</t>
         </is>
       </c>
       <c r="C252" s="15" t="inlineStr">
         <is>
-          <t>SO2609-69603</t>
+          <t>SO2609-68940</t>
         </is>
       </c>
       <c r="D252" s="15" t="n">
-        <v>5100</v>
+        <v>30000</v>
       </c>
       <c r="E252" s="15" t="n">
-        <v>5100</v>
+        <v>30000</v>
       </c>
       <c r="F252" s="15" t="inlineStr">
         <is>
@@ -11300,7 +11300,7 @@
       </c>
       <c r="G252" s="15" t="inlineStr">
         <is>
-          <t>BELGO-MESSASSI</t>
+          <t>BELGO-NKOLBISSON</t>
         </is>
       </c>
       <c r="H252" s="15" t="inlineStr">
@@ -11310,7 +11310,7 @@
       </c>
       <c r="I252" s="15" t="inlineStr">
         <is>
-          <t>16/02/2027</t>
+          <t>17/02/2027</t>
         </is>
       </c>
     </row>
@@ -11322,14 +11322,14 @@
       </c>
       <c r="C253" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68940</t>
+          <t>SO2609-68941</t>
         </is>
       </c>
       <c r="D253" s="15" t="n">
-        <v>30000</v>
+        <v>5000</v>
       </c>
       <c r="E253" s="15" t="n">
-        <v>30000</v>
+        <v>5000</v>
       </c>
       <c r="F253" s="15" t="inlineStr">
         <is>
@@ -11348,35 +11348,35 @@
       </c>
       <c r="I253" s="15" t="inlineStr">
         <is>
-          <t>17/02/2027</t>
+          <t>19/02/2027</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="B254" s="15" t="inlineStr">
         <is>
-          <t>GLOBAL BUSINESS</t>
+          <t>SAGUEN DEFFO CHANCELIER RICHARD</t>
         </is>
       </c>
       <c r="C254" s="15" t="inlineStr">
         <is>
-          <t>SO2609-68941</t>
+          <t>SO2609-69877</t>
         </is>
       </c>
       <c r="D254" s="15" t="n">
-        <v>5000</v>
+        <v>30000</v>
       </c>
       <c r="E254" s="15" t="n">
-        <v>5000</v>
+        <v>30000</v>
       </c>
       <c r="F254" s="15" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="G254" s="15" t="inlineStr">
         <is>
-          <t>BELGO-NKOLBISSON</t>
+          <t>BELGO-FAMLA</t>
         </is>
       </c>
       <c r="H254" s="15" t="inlineStr">
@@ -11385,44 +11385,6 @@
         </is>
       </c>
       <c r="I254" s="15" t="inlineStr">
-        <is>
-          <t>19/02/2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="B255" s="15" t="inlineStr">
-        <is>
-          <t>SAGUEN DEFFO CHANCELIER RICHARD</t>
-        </is>
-      </c>
-      <c r="C255" s="15" t="inlineStr">
-        <is>
-          <t>SO2609-69877</t>
-        </is>
-      </c>
-      <c r="D255" s="15" t="n">
-        <v>30000</v>
-      </c>
-      <c r="E255" s="15" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F255" s="15" t="inlineStr">
-        <is>
-          <t>Ouest</t>
-        </is>
-      </c>
-      <c r="G255" s="15" t="inlineStr">
-        <is>
-          <t>BELGO-FAMLA</t>
-        </is>
-      </c>
-      <c r="H255" s="15" t="inlineStr">
-        <is>
-          <t>NON ÉCHUE</t>
-        </is>
-      </c>
-      <c r="I255" s="15" t="inlineStr">
         <is>
           <t>20/02/2027</t>
         </is>

</xml_diff>